<commit_message>
feat(ui): condition demo video player, split-model pipeline, and misc fixes
- Replace Smokeview launch with in-app mp4 demo playback for the current
  condition (facility + heat source), with Chinese condition info bar,
  play/pause icons and a seek bar
- Resolve demo clips for trained-only facilities via their reference-case
  CHID prefix (agent_damage/cases); rename demo videos to canonical names
- Show the better of cv/holdout grade accuracy as 综合验证准确率
- Silence FFmpeg/QFuture console noise during video playback
- Add per-facility split-model predictor, training and audit scripts;
  Windows packaging files; untrack video/ and presentation/ assets
</commit_message>
<xml_diff>
--- a/export/all_combustibles.xlsx
+++ b/export/all_combustibles.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="所有设施" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="所有设施" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>